<commit_message>
Update Stavfel och språkbruk.xlsx with new analysis data
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$5</definedName>

</xml_diff>

<commit_message>
Update course plans and analysis documents with new data and corrections
- Updated the "Vilande kursplaner.md" file to reflect the current number of problematic course plans, increasing from 3 to 146 findings, and added detailed links for each course plan.
- Updated the "Stavfel och språkbruk.xlsx" file with new data.
- Updated the "Vilande kursplaner.xlsx" file with new data.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,12 +472,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GSQ25F</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -492,19 +492,19 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GSQ2J4</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -519,19 +519,19 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L8</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -546,39 +546,174 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>GSQ25F</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>GSQ25K</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2J4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2L8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>GSQ2PH</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>SQQ</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -588,6 +723,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis documents and Excel files for ISLL and IKS
- Updated download links in markdown files to reflect new file paths for Betygsskalor, Bloom-taxonomi, Examinationsformer, Frasningskonsistens, Omfång, Samstämighet, and Stavfel och språkbruk.
- Replaced old Excel files with new versions for Betygsskalor, Bloom-taxonomi, Examinationsformer, Frasningskonsistens, Omfång, Samstämighet, and Stavfel och språkbruk.
- Adjusted the number of findings displayed in the Stavfel och språkbruk analysis.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$10</definedName>

</xml_diff>

<commit_message>
Update analysis files across multiple departments
- Updated Betygsskalor.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Updated Bloom-taxonomi.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Updated Examinationsformer.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Updated Frasningskonsistens lärandemål.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Updated Omfång på lärandemål.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Updated Samstämmighet svenska och engelska.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Updated Stavfel och språkbruk.md and Stavfel och språkbruk.xlsx in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$10</definedName>

</xml_diff>

<commit_message>
Update analysis files and correct spelling errors in course plans
- Modified multiple Excel files in the "Analys" directory for both IKS and ISLL, addressing discrepancies and updates in data.
- Updated the Markdown file "Stavfel och språkbruk.md" to reflect the latest findings, including a reduction in the number of identified spelling errors from 122 to 5.
- Ensured consistency in file naming and structure across the analysis documents.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,12 +472,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>BY3005</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,24 +487,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>GBY2J2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -514,24 +514,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2J2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>GBY2XF</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -541,12 +541,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2XF</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men delmoment i U,G,VG</t>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -712,8 +712,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>GSQ33M</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33M</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GSQ33N</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -733,6 +787,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis spreadsheet with new data in 'Övrigt.xlsx'
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsskalor.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Betygsskalor" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsskalor'!$A$1:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,14 +432,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,15 +457,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Fastställd</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Reviderad</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Detalj</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Länk</t>
         </is>
@@ -482,15 +494,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+          <t>2017-12-14</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
         </is>
@@ -509,15 +527,21 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+          <t>2020-09-03</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2J2</t>
         </is>
@@ -536,15 +560,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+          <t>2022-09-05</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2XF</t>
         </is>
@@ -563,15 +593,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+          <t>2018-06-14</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
@@ -590,15 +626,21 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+          <t>2018-10-29</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
         </is>
@@ -617,15 +659,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+          <t>2018-11-08</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
@@ -644,15 +692,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
+          <t>2020-09-03</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
         </is>
@@ -671,15 +725,21 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+          <t>2020-12-17</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
         </is>
@@ -698,15 +758,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+          <t>2021-04-15</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
         </is>
@@ -725,15 +791,21 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+          <t>2023-03-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33M</t>
         </is>
@@ -752,45 +824,51 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Inkonsekvent delskalor</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+          <t>2023-03-07</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Inkonsekvent delskalor: kursnivå U,3,4,5 men VG nämns i delmoment</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:G12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>